<commit_message>
feat: implement identity authentication, token rotation, and customer profile APIs
</commit_message>
<xml_diff>
--- a/WebChicKen_WBS_85_Tasks.xlsx
+++ b/WebChicKen_WBS_85_Tasks.xlsx
@@ -287,70 +287,70 @@
     <t>Tạo RegisterRequest, LoginRequest, CreateAddressRequest, UpdateProfileRequest, AuthResponse, UserProfileResponse, AddressResponse trong modules/identity/model/dto/.</t>
   </si>
   <si>
+    <t>TASK-17</t>
+  </si>
+  <si>
+    <t>Hoàn thiện AuthServiceImpl (Đăng ký &amp; Đăng nhập)</t>
+  </si>
+  <si>
+    <t>Logic xác thực tài khoản an toàn với BCrypt và JWT.</t>
+  </si>
+  <si>
+    <t>Trong AuthServiceImpl: register() mã hóa mật khẩu bằng BCrypt, tạo UserEntity và CustomerEntity. login() kiểm tra email, verify BCrypt, check bảng account_bans, sinh JWT và tạo session.</t>
+  </si>
+  <si>
+    <t>TASK-18</t>
+  </si>
+  <si>
+    <t>Hoàn thiện logic Refresh Token xoay vòng (Token Rotation)</t>
+  </si>
+  <si>
+    <t>Thu hồi token và phát hiện tấn công phát lại (Replay Attack).</t>
+  </si>
+  <si>
+    <t>Tìm session trong user_sessions. Nếu token đã thu hồi/đã dùng, xóa sạch mọi session của user đó. Nếu hợp lệ, revoke token cũ, sinh cặp token mới và cập nhật DB.</t>
+  </si>
+  <si>
+    <t>TASK-19</t>
+  </si>
+  <si>
+    <t>Hoàn thiện CustomerServiceImpl và Sổ địa chỉ</t>
+  </si>
+  <si>
+    <t>CRUD sổ địa chỉ giao hàng của người mua.</t>
+  </si>
+  <si>
+    <t>Trong CustomerServiceImpl: Thêm địa chỉ mới, sửa, xóa. Khi một địa chỉ có is_default=true, tự động cập nhật các địa chỉ còn lại của user về false.</t>
+  </si>
+  <si>
+    <t>TASK-20</t>
+  </si>
+  <si>
+    <t>Hoàn thiện AuthServlet và CustomerServlet</t>
+  </si>
+  <si>
+    <t>Tiếp nhận HTTP request, validate cơ bản và ủy quyền cho Service.</t>
+  </si>
+  <si>
+    <t>Kế thừa BaseApiServlet, xử lý /login, /register, /refresh, /logout, /addresses. Ghi cookie HttpOnly cho refresh token; trả access token trong body JSON.</t>
+  </si>
+  <si>
+    <t>TASK-21</t>
+  </si>
+  <si>
+    <t>Frontend Auth</t>
+  </si>
+  <si>
+    <t>Xây dựng màn hình Đăng ký / Đăng nhập phía Frontend</t>
+  </si>
+  <si>
+    <t>Form xác thực có validate trực quan, xử lý trạng thái loading và thông báo lỗi.</t>
+  </si>
+  <si>
+    <t>Trong features/auth/: Viết schema Zod loginSchema, registerSchema. Dùng React Hook Form. Lưu token vào authStore và điều hướng về trang trước đó hoặc trang chủ.</t>
+  </si>
+  <si>
     <t>☐ CHƯA XONG</t>
-  </si>
-  <si>
-    <t>TASK-17</t>
-  </si>
-  <si>
-    <t>Hoàn thiện AuthServiceImpl (Đăng ký &amp; Đăng nhập)</t>
-  </si>
-  <si>
-    <t>Logic xác thực tài khoản an toàn với BCrypt và JWT.</t>
-  </si>
-  <si>
-    <t>Trong AuthServiceImpl: register() mã hóa mật khẩu bằng BCrypt, tạo UserEntity và CustomerEntity. login() kiểm tra email, verify BCrypt, check bảng account_bans, sinh JWT và tạo session.</t>
-  </si>
-  <si>
-    <t>TASK-18</t>
-  </si>
-  <si>
-    <t>Hoàn thiện logic Refresh Token xoay vòng (Token Rotation)</t>
-  </si>
-  <si>
-    <t>Thu hồi token và phát hiện tấn công phát lại (Replay Attack).</t>
-  </si>
-  <si>
-    <t>Tìm session trong user_sessions. Nếu token đã thu hồi/đã dùng, xóa sạch mọi session của user đó. Nếu hợp lệ, revoke token cũ, sinh cặp token mới và cập nhật DB.</t>
-  </si>
-  <si>
-    <t>TASK-19</t>
-  </si>
-  <si>
-    <t>Hoàn thiện CustomerServiceImpl và Sổ địa chỉ</t>
-  </si>
-  <si>
-    <t>CRUD sổ địa chỉ giao hàng của người mua.</t>
-  </si>
-  <si>
-    <t>Trong CustomerServiceImpl: Thêm địa chỉ mới, sửa, xóa. Khi một địa chỉ có is_default=true, tự động cập nhật các địa chỉ còn lại của user về false.</t>
-  </si>
-  <si>
-    <t>TASK-20</t>
-  </si>
-  <si>
-    <t>Hoàn thiện AuthServlet và CustomerServlet</t>
-  </si>
-  <si>
-    <t>Tiếp nhận HTTP request, validate cơ bản và ủy quyền cho Service.</t>
-  </si>
-  <si>
-    <t>Kế thừa BaseApiServlet, xử lý /login, /register, /refresh, /logout, /addresses. Ghi cookie HttpOnly cho refresh token; trả access token trong body JSON.</t>
-  </si>
-  <si>
-    <t>TASK-21</t>
-  </si>
-  <si>
-    <t>Frontend Auth</t>
-  </si>
-  <si>
-    <t>Xây dựng màn hình Đăng ký / Đăng nhập phía Frontend</t>
-  </si>
-  <si>
-    <t>Form xác thực có validate trực quan, xử lý trạng thái loading và thông báo lỗi.</t>
-  </si>
-  <si>
-    <t>Trong features/auth/: Viết schema Zod loginSchema, registerSchema. Dùng React Hook Form. Lưu token vào authStore và điều hướng về trang trước đó hoặc trang chủ.</t>
   </si>
   <si>
     <t>TASK-22</t>
@@ -1269,7 +1269,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1316,6 +1316,7 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF16A34A"/>
       <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
@@ -1329,6 +1330,11 @@
       <b/>
       <color rgb="FF64748B"/>
       <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
     <font>
@@ -1514,14 +1520,14 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1529,10 +1535,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2452,7 +2458,7 @@
         <v>90</v>
       </c>
       <c r="I18" s="17" t="s">
-        <v>91</v>
+        <v>19</v>
       </c>
       <c r="J18" s="18">
         <f>IF(I18="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2460,7 +2466,7 @@
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>86</v>
@@ -2469,7 +2475,7 @@
         <v>87</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>15</v>
@@ -2478,13 +2484,13 @@
         <v>16</v>
       </c>
       <c r="G19" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H19" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="H19" s="8" t="s">
-        <v>95</v>
-      </c>
       <c r="I19" s="9" t="s">
-        <v>91</v>
+        <v>19</v>
       </c>
       <c r="J19" s="10">
         <f>IF(I19="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2492,7 +2498,7 @@
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>86</v>
@@ -2501,7 +2507,7 @@
         <v>87</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>15</v>
@@ -2510,13 +2516,13 @@
         <v>16</v>
       </c>
       <c r="G20" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="H20" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="H20" s="16" t="s">
-        <v>99</v>
-      </c>
       <c r="I20" s="17" t="s">
-        <v>91</v>
+        <v>19</v>
       </c>
       <c r="J20" s="18">
         <f>IF(I20="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2524,7 +2530,7 @@
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>86</v>
@@ -2533,7 +2539,7 @@
         <v>87</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>15</v>
@@ -2542,13 +2548,13 @@
         <v>43</v>
       </c>
       <c r="G21" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="H21" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="H21" s="8" t="s">
-        <v>103</v>
-      </c>
       <c r="I21" s="9" t="s">
-        <v>91</v>
+        <v>19</v>
       </c>
       <c r="J21" s="10">
         <f>IF(I21="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2556,7 +2562,7 @@
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>86</v>
@@ -2565,7 +2571,7 @@
         <v>87</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>15</v>
@@ -2574,13 +2580,13 @@
         <v>16</v>
       </c>
       <c r="G22" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="H22" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="H22" s="16" t="s">
-        <v>107</v>
-      </c>
       <c r="I22" s="17" t="s">
-        <v>91</v>
+        <v>19</v>
       </c>
       <c r="J22" s="18">
         <f>IF(I22="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2588,16 +2594,16 @@
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>86</v>
       </c>
       <c r="C23" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>74</v>
@@ -2606,13 +2612,13 @@
         <v>16</v>
       </c>
       <c r="G23" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="H23" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="H23" s="8" t="s">
-        <v>112</v>
-      </c>
       <c r="I23" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J23" s="10">
         <f>IF(I23="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2644,7 +2650,7 @@
         <v>117</v>
       </c>
       <c r="I24" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J24" s="18">
         <f>IF(I24="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2676,7 +2682,7 @@
         <v>122</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J25" s="10">
         <f>IF(I25="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2708,7 +2714,7 @@
         <v>126</v>
       </c>
       <c r="I26" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J26" s="18">
         <f>IF(I26="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2740,7 +2746,7 @@
         <v>131</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J27" s="10">
         <f>IF(I27="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2772,7 +2778,7 @@
         <v>136</v>
       </c>
       <c r="I28" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J28" s="18">
         <f>IF(I28="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2804,7 +2810,7 @@
         <v>141</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J29" s="10">
         <f>IF(I29="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2836,7 +2842,7 @@
         <v>145</v>
       </c>
       <c r="I30" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J30" s="18">
         <f>IF(I30="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2868,7 +2874,7 @@
         <v>149</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J31" s="10">
         <f>IF(I31="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2900,7 +2906,7 @@
         <v>153</v>
       </c>
       <c r="I32" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J32" s="18">
         <f>IF(I32="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2932,7 +2938,7 @@
         <v>158</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J33" s="10">
         <f>IF(I33="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2964,7 +2970,7 @@
         <v>163</v>
       </c>
       <c r="I34" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J34" s="18">
         <f>IF(I34="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2996,7 +3002,7 @@
         <v>167</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J35" s="10">
         <f>IF(I35="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3028,7 +3034,7 @@
         <v>172</v>
       </c>
       <c r="I36" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J36" s="18">
         <f>IF(I36="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3060,7 +3066,7 @@
         <v>176</v>
       </c>
       <c r="I37" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J37" s="10">
         <f>IF(I37="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3092,7 +3098,7 @@
         <v>182</v>
       </c>
       <c r="I38" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J38" s="18">
         <f>IF(I38="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3124,7 +3130,7 @@
         <v>186</v>
       </c>
       <c r="I39" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J39" s="10">
         <f>IF(I39="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3156,7 +3162,7 @@
         <v>191</v>
       </c>
       <c r="I40" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J40" s="18">
         <f>IF(I40="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3188,7 +3194,7 @@
         <v>195</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J41" s="10">
         <f>IF(I41="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3220,7 +3226,7 @@
         <v>199</v>
       </c>
       <c r="I42" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J42" s="18">
         <f>IF(I42="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3252,7 +3258,7 @@
         <v>204</v>
       </c>
       <c r="I43" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J43" s="10">
         <f>IF(I43="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3284,7 +3290,7 @@
         <v>209</v>
       </c>
       <c r="I44" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J44" s="18">
         <f>IF(I44="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3316,7 +3322,7 @@
         <v>214</v>
       </c>
       <c r="I45" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J45" s="10">
         <f>IF(I45="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3348,7 +3354,7 @@
         <v>219</v>
       </c>
       <c r="I46" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J46" s="18">
         <f>IF(I46="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3380,7 +3386,7 @@
         <v>223</v>
       </c>
       <c r="I47" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J47" s="10">
         <f>IF(I47="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3412,7 +3418,7 @@
         <v>227</v>
       </c>
       <c r="I48" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J48" s="18">
         <f>IF(I48="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3444,7 +3450,7 @@
         <v>232</v>
       </c>
       <c r="I49" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J49" s="10">
         <f>IF(I49="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3476,7 +3482,7 @@
         <v>237</v>
       </c>
       <c r="I50" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J50" s="18">
         <f>IF(I50="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3508,7 +3514,7 @@
         <v>241</v>
       </c>
       <c r="I51" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J51" s="10">
         <f>IF(I51="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3540,7 +3546,7 @@
         <v>246</v>
       </c>
       <c r="I52" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J52" s="18">
         <f>IF(I52="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3572,7 +3578,7 @@
         <v>250</v>
       </c>
       <c r="I53" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J53" s="10">
         <f>IF(I53="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3604,7 +3610,7 @@
         <v>254</v>
       </c>
       <c r="I54" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J54" s="18">
         <f>IF(I54="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3636,7 +3642,7 @@
         <v>259</v>
       </c>
       <c r="I55" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J55" s="10">
         <f>IF(I55="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3668,7 +3674,7 @@
         <v>263</v>
       </c>
       <c r="I56" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J56" s="18">
         <f>IF(I56="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3700,7 +3706,7 @@
         <v>268</v>
       </c>
       <c r="I57" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J57" s="10">
         <f>IF(I57="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3732,7 +3738,7 @@
         <v>274</v>
       </c>
       <c r="I58" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J58" s="18">
         <f>IF(I58="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3764,7 +3770,7 @@
         <v>278</v>
       </c>
       <c r="I59" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J59" s="10">
         <f>IF(I59="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3796,7 +3802,7 @@
         <v>282</v>
       </c>
       <c r="I60" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J60" s="18">
         <f>IF(I60="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3828,7 +3834,7 @@
         <v>287</v>
       </c>
       <c r="I61" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J61" s="10">
         <f>IF(I61="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3860,7 +3866,7 @@
         <v>291</v>
       </c>
       <c r="I62" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J62" s="18">
         <f>IF(I62="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3892,7 +3898,7 @@
         <v>295</v>
       </c>
       <c r="I63" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J63" s="10">
         <f>IF(I63="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3924,7 +3930,7 @@
         <v>299</v>
       </c>
       <c r="I64" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J64" s="18">
         <f>IF(I64="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3956,7 +3962,7 @@
         <v>304</v>
       </c>
       <c r="I65" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J65" s="10">
         <f>IF(I65="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3988,7 +3994,7 @@
         <v>308</v>
       </c>
       <c r="I66" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J66" s="18">
         <f>IF(I66="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4020,7 +4026,7 @@
         <v>312</v>
       </c>
       <c r="I67" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J67" s="10">
         <f>IF(I67="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4052,7 +4058,7 @@
         <v>316</v>
       </c>
       <c r="I68" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J68" s="18">
         <f>IF(I68="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4084,7 +4090,7 @@
         <v>320</v>
       </c>
       <c r="I69" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J69" s="10">
         <f>IF(I69="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4116,7 +4122,7 @@
         <v>325</v>
       </c>
       <c r="I70" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J70" s="18">
         <f>IF(I70="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4148,7 +4154,7 @@
         <v>330</v>
       </c>
       <c r="I71" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J71" s="10">
         <f>IF(I71="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4180,7 +4186,7 @@
         <v>334</v>
       </c>
       <c r="I72" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J72" s="18">
         <f>IF(I72="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4212,7 +4218,7 @@
         <v>341</v>
       </c>
       <c r="I73" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J73" s="10">
         <f>IF(I73="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4244,7 +4250,7 @@
         <v>345</v>
       </c>
       <c r="I74" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J74" s="18">
         <f>IF(I74="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4276,7 +4282,7 @@
         <v>349</v>
       </c>
       <c r="I75" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J75" s="10">
         <f>IF(I75="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4308,7 +4314,7 @@
         <v>353</v>
       </c>
       <c r="I76" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J76" s="18">
         <f>IF(I76="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4340,7 +4346,7 @@
         <v>357</v>
       </c>
       <c r="I77" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J77" s="10">
         <f>IF(I77="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4372,7 +4378,7 @@
         <v>361</v>
       </c>
       <c r="I78" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J78" s="18">
         <f>IF(I78="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4404,7 +4410,7 @@
         <v>365</v>
       </c>
       <c r="I79" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J79" s="10">
         <f>IF(I79="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4436,7 +4442,7 @@
         <v>370</v>
       </c>
       <c r="I80" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J80" s="18">
         <f>IF(I80="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4468,7 +4474,7 @@
         <v>375</v>
       </c>
       <c r="I81" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J81" s="10">
         <f>IF(I81="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4500,7 +4506,7 @@
         <v>380</v>
       </c>
       <c r="I82" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J82" s="18">
         <f>IF(I82="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4532,7 +4538,7 @@
         <v>386</v>
       </c>
       <c r="I83" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J83" s="10">
         <f>IF(I83="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4564,7 +4570,7 @@
         <v>390</v>
       </c>
       <c r="I84" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J84" s="18">
         <f>IF(I84="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4596,7 +4602,7 @@
         <v>394</v>
       </c>
       <c r="I85" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J85" s="10">
         <f>IF(I85="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4628,7 +4634,7 @@
         <v>398</v>
       </c>
       <c r="I86" s="17" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J86" s="18">
         <f>IF(I86="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4660,7 +4666,7 @@
         <v>404</v>
       </c>
       <c r="I87" s="9" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="J87" s="10">
         <f>IF(I87="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>

</xml_diff>

<commit_message>
feat: implement modern marketplace authentication UI and routing
</commit_message>
<xml_diff>
--- a/WebChicKen_WBS_85_Tasks.xlsx
+++ b/WebChicKen_WBS_85_Tasks.xlsx
@@ -350,22 +350,22 @@
     <t>Trong features/auth/: Viết schema Zod loginSchema, registerSchema. Dùng React Hook Form. Lưu token vào authStore và điều hướng về trang trước đó hoặc trang chủ.</t>
   </si>
   <si>
+    <t>TASK-22</t>
+  </si>
+  <si>
+    <t>Frontend Account</t>
+  </si>
+  <si>
+    <t>Xây dựng màn hình Quản lý Hồ sơ &amp; Sổ địa chỉ</t>
+  </si>
+  <si>
+    <t>Người mua xem/sửa thông tin cá nhân và thiết lập địa chỉ nhận hàng mặc định.</t>
+  </si>
+  <si>
+    <t>Trong pages/buyer/account/: Viết AddressCard, Modal thêm/sửa địa chỉ, tích hợp danh sách Tỉnh/Thành, Quận/Huyện, Phường/Xã.</t>
+  </si>
+  <si>
     <t>☐ CHƯA XONG</t>
-  </si>
-  <si>
-    <t>TASK-22</t>
-  </si>
-  <si>
-    <t>Frontend Account</t>
-  </si>
-  <si>
-    <t>Xây dựng màn hình Quản lý Hồ sơ &amp; Sổ địa chỉ</t>
-  </si>
-  <si>
-    <t>Người mua xem/sửa thông tin cá nhân và thiết lập địa chỉ nhận hàng mặc định.</t>
-  </si>
-  <si>
-    <t>Trong pages/buyer/account/: Viết AddressCard, Modal thêm/sửa địa chỉ, tích hợp danh sách Tỉnh/Thành, Quận/Huyện, Phường/Xã.</t>
   </si>
   <si>
     <t>TASK-23</t>
@@ -2618,7 +2618,7 @@
         <v>111</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>112</v>
+        <v>19</v>
       </c>
       <c r="J23" s="10">
         <f>IF(I23="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2626,16 +2626,16 @@
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>86</v>
       </c>
       <c r="C24" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" s="14" t="s">
         <v>114</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>115</v>
       </c>
       <c r="E24" s="13" t="s">
         <v>74</v>
@@ -2644,13 +2644,13 @@
         <v>43</v>
       </c>
       <c r="G24" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="H24" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="H24" s="16" t="s">
-        <v>117</v>
-      </c>
       <c r="I24" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J24" s="18">
         <f>IF(I24="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2682,7 +2682,7 @@
         <v>122</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J25" s="10">
         <f>IF(I25="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2714,7 +2714,7 @@
         <v>126</v>
       </c>
       <c r="I26" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J26" s="18">
         <f>IF(I26="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2746,7 +2746,7 @@
         <v>131</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J27" s="10">
         <f>IF(I27="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2778,7 +2778,7 @@
         <v>136</v>
       </c>
       <c r="I28" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J28" s="18">
         <f>IF(I28="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2810,7 +2810,7 @@
         <v>141</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J29" s="10">
         <f>IF(I29="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2842,7 +2842,7 @@
         <v>145</v>
       </c>
       <c r="I30" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J30" s="18">
         <f>IF(I30="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2874,7 +2874,7 @@
         <v>149</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J31" s="10">
         <f>IF(I31="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2906,7 +2906,7 @@
         <v>153</v>
       </c>
       <c r="I32" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J32" s="18">
         <f>IF(I32="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2938,7 +2938,7 @@
         <v>158</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J33" s="10">
         <f>IF(I33="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2970,7 +2970,7 @@
         <v>163</v>
       </c>
       <c r="I34" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J34" s="18">
         <f>IF(I34="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3002,7 +3002,7 @@
         <v>167</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J35" s="10">
         <f>IF(I35="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3034,7 +3034,7 @@
         <v>172</v>
       </c>
       <c r="I36" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J36" s="18">
         <f>IF(I36="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3066,7 +3066,7 @@
         <v>176</v>
       </c>
       <c r="I37" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J37" s="10">
         <f>IF(I37="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3098,7 +3098,7 @@
         <v>182</v>
       </c>
       <c r="I38" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J38" s="18">
         <f>IF(I38="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3130,7 +3130,7 @@
         <v>186</v>
       </c>
       <c r="I39" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J39" s="10">
         <f>IF(I39="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3162,7 +3162,7 @@
         <v>191</v>
       </c>
       <c r="I40" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J40" s="18">
         <f>IF(I40="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3194,7 +3194,7 @@
         <v>195</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J41" s="10">
         <f>IF(I41="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3226,7 +3226,7 @@
         <v>199</v>
       </c>
       <c r="I42" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J42" s="18">
         <f>IF(I42="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3258,7 +3258,7 @@
         <v>204</v>
       </c>
       <c r="I43" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J43" s="10">
         <f>IF(I43="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3290,7 +3290,7 @@
         <v>209</v>
       </c>
       <c r="I44" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J44" s="18">
         <f>IF(I44="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3322,7 +3322,7 @@
         <v>214</v>
       </c>
       <c r="I45" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J45" s="10">
         <f>IF(I45="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3354,7 +3354,7 @@
         <v>219</v>
       </c>
       <c r="I46" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J46" s="18">
         <f>IF(I46="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3386,7 +3386,7 @@
         <v>223</v>
       </c>
       <c r="I47" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J47" s="10">
         <f>IF(I47="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3418,7 +3418,7 @@
         <v>227</v>
       </c>
       <c r="I48" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J48" s="18">
         <f>IF(I48="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3450,7 +3450,7 @@
         <v>232</v>
       </c>
       <c r="I49" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J49" s="10">
         <f>IF(I49="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3482,7 +3482,7 @@
         <v>237</v>
       </c>
       <c r="I50" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J50" s="18">
         <f>IF(I50="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3514,7 +3514,7 @@
         <v>241</v>
       </c>
       <c r="I51" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J51" s="10">
         <f>IF(I51="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3546,7 +3546,7 @@
         <v>246</v>
       </c>
       <c r="I52" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J52" s="18">
         <f>IF(I52="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3578,7 +3578,7 @@
         <v>250</v>
       </c>
       <c r="I53" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J53" s="10">
         <f>IF(I53="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3610,7 +3610,7 @@
         <v>254</v>
       </c>
       <c r="I54" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J54" s="18">
         <f>IF(I54="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3642,7 +3642,7 @@
         <v>259</v>
       </c>
       <c r="I55" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J55" s="10">
         <f>IF(I55="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3674,7 +3674,7 @@
         <v>263</v>
       </c>
       <c r="I56" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J56" s="18">
         <f>IF(I56="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3706,7 +3706,7 @@
         <v>268</v>
       </c>
       <c r="I57" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J57" s="10">
         <f>IF(I57="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3738,7 +3738,7 @@
         <v>274</v>
       </c>
       <c r="I58" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J58" s="18">
         <f>IF(I58="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3770,7 +3770,7 @@
         <v>278</v>
       </c>
       <c r="I59" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J59" s="10">
         <f>IF(I59="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3802,7 +3802,7 @@
         <v>282</v>
       </c>
       <c r="I60" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J60" s="18">
         <f>IF(I60="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3834,7 +3834,7 @@
         <v>287</v>
       </c>
       <c r="I61" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J61" s="10">
         <f>IF(I61="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3866,7 +3866,7 @@
         <v>291</v>
       </c>
       <c r="I62" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J62" s="18">
         <f>IF(I62="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3898,7 +3898,7 @@
         <v>295</v>
       </c>
       <c r="I63" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J63" s="10">
         <f>IF(I63="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3930,7 +3930,7 @@
         <v>299</v>
       </c>
       <c r="I64" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J64" s="18">
         <f>IF(I64="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3962,7 +3962,7 @@
         <v>304</v>
       </c>
       <c r="I65" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J65" s="10">
         <f>IF(I65="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3994,7 +3994,7 @@
         <v>308</v>
       </c>
       <c r="I66" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J66" s="18">
         <f>IF(I66="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4026,7 +4026,7 @@
         <v>312</v>
       </c>
       <c r="I67" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J67" s="10">
         <f>IF(I67="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4058,7 +4058,7 @@
         <v>316</v>
       </c>
       <c r="I68" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J68" s="18">
         <f>IF(I68="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4090,7 +4090,7 @@
         <v>320</v>
       </c>
       <c r="I69" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J69" s="10">
         <f>IF(I69="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4122,7 +4122,7 @@
         <v>325</v>
       </c>
       <c r="I70" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J70" s="18">
         <f>IF(I70="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4154,7 +4154,7 @@
         <v>330</v>
       </c>
       <c r="I71" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J71" s="10">
         <f>IF(I71="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4186,7 +4186,7 @@
         <v>334</v>
       </c>
       <c r="I72" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J72" s="18">
         <f>IF(I72="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4218,7 +4218,7 @@
         <v>341</v>
       </c>
       <c r="I73" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J73" s="10">
         <f>IF(I73="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4250,7 +4250,7 @@
         <v>345</v>
       </c>
       <c r="I74" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J74" s="18">
         <f>IF(I74="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4282,7 +4282,7 @@
         <v>349</v>
       </c>
       <c r="I75" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J75" s="10">
         <f>IF(I75="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4314,7 +4314,7 @@
         <v>353</v>
       </c>
       <c r="I76" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J76" s="18">
         <f>IF(I76="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4346,7 +4346,7 @@
         <v>357</v>
       </c>
       <c r="I77" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J77" s="10">
         <f>IF(I77="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4378,7 +4378,7 @@
         <v>361</v>
       </c>
       <c r="I78" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J78" s="18">
         <f>IF(I78="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4410,7 +4410,7 @@
         <v>365</v>
       </c>
       <c r="I79" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J79" s="10">
         <f>IF(I79="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4442,7 +4442,7 @@
         <v>370</v>
       </c>
       <c r="I80" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J80" s="18">
         <f>IF(I80="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4474,7 +4474,7 @@
         <v>375</v>
       </c>
       <c r="I81" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J81" s="10">
         <f>IF(I81="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4506,7 +4506,7 @@
         <v>380</v>
       </c>
       <c r="I82" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J82" s="18">
         <f>IF(I82="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4538,7 +4538,7 @@
         <v>386</v>
       </c>
       <c r="I83" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J83" s="10">
         <f>IF(I83="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4570,7 +4570,7 @@
         <v>390</v>
       </c>
       <c r="I84" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J84" s="18">
         <f>IF(I84="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4602,7 +4602,7 @@
         <v>394</v>
       </c>
       <c r="I85" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J85" s="10">
         <f>IF(I85="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4634,7 +4634,7 @@
         <v>398</v>
       </c>
       <c r="I86" s="17" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J86" s="18">
         <f>IF(I86="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4666,7 +4666,7 @@
         <v>404</v>
       </c>
       <c r="I87" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J87" s="10">
         <f>IF(I87="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>

</xml_diff>

<commit_message>
feat(marketplace): implement inventory reservation, cart sync, voucher engine, multi-shop checkout, and orders management
</commit_message>
<xml_diff>
--- a/WebChicKen_WBS_85_Tasks.xlsx
+++ b/WebChicKen_WBS_85_Tasks.xlsx
@@ -1,17 +1,49 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
-  <sheets>
-    <sheet sheetId="1" name="WBS - 85 Tasks Backlog" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Thống kê Tiến độ (Dashboard)" state="visible" r:id="rId5"/>
-  </sheets>
-  <calcPr calcId="171027"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>2</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="2" baseType="lpstr">
+      <vt:lpstr>WBS - 85 Tasks Backlog</vt:lpstr>
+      <vt:lpstr>Thống kê Tiến độ (Dashboard)</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <Manager/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Antigravity IDE - Tech Lead</dc:creator>
+  <dc:title/>
+  <dc:subject/>
+  <dc:description/>
+  <cp:keywords/>
+  <cp:category/>
+  <cp:lastModifiedBy>Unknown</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-10-01T15:47:08Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-10-01T15:47:08Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="416">
   <si>
     <t>DỰ ÁN WEBCHICKEN E-COMMERCE — BẢN PHÂN RÃ CÔNG VIỆC (WBS 85 TASKS BACKLOG)</t>
@@ -1264,7 +1296,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
@@ -1569,7 +1601,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1889,7 +1921,19 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <sheets>
+    <sheet sheetId="1" name="WBS - 85 Tasks Backlog" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Thống kê Tiến độ (Dashboard)" state="visible" r:id="rId5"/>
+  </sheets>
+  <calcPr calcId="171027"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J87"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2649,8 +2693,8 @@
       <c r="H24" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="I24" s="17" t="s">
-        <v>117</v>
+      <c r="I24" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J24" s="18">
         <f>IF(I24="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2682,7 +2726,7 @@
         <v>122</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J25" s="10">
         <f>IF(I25="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2713,8 +2757,8 @@
       <c r="H26" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="I26" s="17" t="s">
-        <v>117</v>
+      <c r="I26" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J26" s="18">
         <f>IF(I26="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2746,7 +2790,7 @@
         <v>131</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J27" s="10">
         <f>IF(I27="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2777,8 +2821,8 @@
       <c r="H28" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="I28" s="17" t="s">
-        <v>117</v>
+      <c r="I28" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J28" s="18">
         <f>IF(I28="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2810,7 +2854,7 @@
         <v>141</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J29" s="10">
         <f>IF(I29="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2841,8 +2885,8 @@
       <c r="H30" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="I30" s="17" t="s">
-        <v>117</v>
+      <c r="I30" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J30" s="18">
         <f>IF(I30="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2874,7 +2918,7 @@
         <v>149</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J31" s="10">
         <f>IF(I31="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2905,8 +2949,8 @@
       <c r="H32" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="I32" s="17" t="s">
-        <v>117</v>
+      <c r="I32" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J32" s="18">
         <f>IF(I32="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2938,7 +2982,7 @@
         <v>158</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J33" s="10">
         <f>IF(I33="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -2969,8 +3013,8 @@
       <c r="H34" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="I34" s="17" t="s">
-        <v>117</v>
+      <c r="I34" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J34" s="18">
         <f>IF(I34="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3002,7 +3046,7 @@
         <v>167</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J35" s="10">
         <f>IF(I35="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3033,8 +3077,8 @@
       <c r="H36" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="I36" s="17" t="s">
-        <v>117</v>
+      <c r="I36" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J36" s="18">
         <f>IF(I36="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3066,7 +3110,7 @@
         <v>176</v>
       </c>
       <c r="I37" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J37" s="10">
         <f>IF(I37="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3097,8 +3141,8 @@
       <c r="H38" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="I38" s="17" t="s">
-        <v>117</v>
+      <c r="I38" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J38" s="18">
         <f>IF(I38="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3130,7 +3174,7 @@
         <v>186</v>
       </c>
       <c r="I39" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J39" s="10">
         <f>IF(I39="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3161,8 +3205,8 @@
       <c r="H40" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="I40" s="17" t="s">
-        <v>117</v>
+      <c r="I40" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J40" s="18">
         <f>IF(I40="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3194,7 +3238,7 @@
         <v>195</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J41" s="10">
         <f>IF(I41="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3225,8 +3269,8 @@
       <c r="H42" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="I42" s="17" t="s">
-        <v>117</v>
+      <c r="I42" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J42" s="18">
         <f>IF(I42="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3258,7 +3302,7 @@
         <v>204</v>
       </c>
       <c r="I43" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J43" s="10">
         <f>IF(I43="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3289,8 +3333,8 @@
       <c r="H44" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="I44" s="17" t="s">
-        <v>117</v>
+      <c r="I44" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J44" s="18">
         <f>IF(I44="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3322,7 +3366,7 @@
         <v>214</v>
       </c>
       <c r="I45" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J45" s="10">
         <f>IF(I45="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3353,8 +3397,8 @@
       <c r="H46" s="16" t="s">
         <v>219</v>
       </c>
-      <c r="I46" s="17" t="s">
-        <v>117</v>
+      <c r="I46" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J46" s="18">
         <f>IF(I46="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3386,7 +3430,7 @@
         <v>223</v>
       </c>
       <c r="I47" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J47" s="10">
         <f>IF(I47="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3417,8 +3461,8 @@
       <c r="H48" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="I48" s="17" t="s">
-        <v>117</v>
+      <c r="I48" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J48" s="18">
         <f>IF(I48="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3450,7 +3494,7 @@
         <v>232</v>
       </c>
       <c r="I49" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J49" s="10">
         <f>IF(I49="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3481,8 +3525,8 @@
       <c r="H50" s="16" t="s">
         <v>237</v>
       </c>
-      <c r="I50" s="17" t="s">
-        <v>117</v>
+      <c r="I50" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="J50" s="18">
         <f>IF(I50="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -3514,7 +3558,7 @@
         <v>241</v>
       </c>
       <c r="I51" s="9" t="s">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="J51" s="10">
         <f>IF(I51="✓ ĐÃ XONG","Hoàn thành","Đang chờ")</f>
@@ -4695,7 +4739,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>

</xml_diff>